<commit_message>
casas particulares: noviembre y diciembre con los anexos rectificados por la Res. CNTCP 7/2026 (1,6%, no 1,7%)
La 6/2026 citó dos anexos equivocados; el cargado el 15/9 subía 1,7% y la página lo publicaba
como 'discrepancia'. La 7/2026 (B.O. 18/9) los corrigió: los 18 valores de cada mes reproducen
(octubre + $5.000) x 1,016 y noviembre x 1,016 al centavo. Lo detectó el semáforo del workflow
datos-vivos en su primera corrida en la nube. El rastreador ahora cuenta las rectificaciones ya
cargadas y el mes vigente usa el mismo reloj (hoyAR) que el resto del sitio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-casas-particulares-2026.xlsx
+++ b/private/planilla-casas-particulares-2026.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="183">
   <si>
     <t>Cómo usar esta planilla</t>
   </si>
@@ -88,7 +88,7 @@
     <t>Sueldo del mes — Personal de Casas Particulares</t>
   </si>
   <si>
-    <t>Ley 26.844 · Resolución CNTCP 6/2026 · Verificado el 2026-09-15</t>
+    <t>Ley 26.844 · Resolución CNTCP 6/2026 · Verificado el 2026-09-28</t>
   </si>
   <si>
     <t>DATOS DEL MES</t>
@@ -427,7 +427,7 @@
     <t>Valores sin zona desfavorable. El adicional del 31% lo aplica el Liquidador. Los caseros solo existen en la modalidad sin retiro (el anexo trae un guion en «con retiro»).</t>
   </si>
   <si>
-    <t>Importes transcriptos de los Anexos 1 a 5 de la Resolución CNTCP 6/2026 (B.O. 3/9/2026), verificados el 2026-09-15. La columna «Clave» la usa el Liquidador: no la borres.</t>
+    <t>Importes transcriptos de los Anexos 1 a 5 de la Resolución CNTCP 6/2026 (B.O. 3/9/2026), verificados el 2026-09-28. La columna «Clave» la usa el Liquidador: no la borres.</t>
   </si>
   <si>
     <t>Aportes, contribuciones y ART — valores de agosto de 2026 (se pagan en septiembre de 2026)</t>
@@ -505,13 +505,19 @@
     <t>Fuentes oficiales</t>
   </si>
   <si>
-    <t>Todos los datos de esta planilla se verificaron el 2026-09-15 contra los documentos oficiales de abajo. Ningún blog, ningún resumen de terceros.</t>
+    <t>Todos los datos de esta planilla se verificaron el 2026-09-28 contra los documentos oficiales de abajo. Ningún blog, ningún resumen de terceros.</t>
   </si>
   <si>
     <t>Documento</t>
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>Resolución CNTCP 7/2026 — rectifica los Anexos 4 y 5 (noviembre y diciembre)</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/347648/20260918</t>
   </si>
   <si>
     <t>Resolución CNTCP 6/2026 (texto completo)</t>
@@ -2110,10 +2116,10 @@
         <v>4805.82</v>
       </c>
       <c r="H3" s="33">
-        <v>4928.28</v>
+        <v>4923.44</v>
       </c>
       <c r="I3" s="33">
-        <v>5007.14</v>
+        <v>5002.21</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -2139,10 +2145,10 @@
         <v>599514.52</v>
       </c>
       <c r="H4" s="36">
-        <v>614791.27</v>
+        <v>614186.76</v>
       </c>
       <c r="I4" s="36">
-        <v>624627.93</v>
+        <v>624013.75</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -2168,10 +2174,10 @@
         <v>5215.59</v>
       </c>
       <c r="H5" s="33">
-        <v>5344.33</v>
+        <v>5339.08</v>
       </c>
       <c r="I5" s="33">
-        <v>5429.84</v>
+        <v>5424.5</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -2197,10 +2203,10 @@
         <v>661702.46</v>
       </c>
       <c r="H6" s="36">
-        <v>678036.4</v>
+        <v>677369.7</v>
       </c>
       <c r="I6" s="36">
-        <v>688884.98</v>
+        <v>688207.61</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -2226,10 +2232,10 @@
         <v>4580.8</v>
       </c>
       <c r="H7" s="33">
-        <v>4700.21</v>
+        <v>4695.59</v>
       </c>
       <c r="I7" s="33">
-        <v>4775.41</v>
+        <v>4770.72</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2255,10 +2261,10 @@
         <v>560776.33</v>
       </c>
       <c r="H8" s="36">
-        <v>575394.53</v>
+        <v>574828.75</v>
       </c>
       <c r="I8" s="36">
-        <v>584600.84</v>
+        <v>584026.01</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -2284,10 +2290,10 @@
         <v>4973.38</v>
       </c>
       <c r="H9" s="33">
-        <v>5098.84</v>
+        <v>5093.82</v>
       </c>
       <c r="I9" s="33">
-        <v>5180.42</v>
+        <v>5175.33</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -2313,10 +2319,10 @@
         <v>618187.89</v>
       </c>
       <c r="H10" s="36">
-        <v>633782.08</v>
+        <v>633158.89</v>
       </c>
       <c r="I10" s="36">
-        <v>643922.59</v>
+        <v>643289.43</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -2380,10 +2386,10 @@
         <v>4337.53</v>
       </c>
       <c r="H13" s="33">
-        <v>4451.49</v>
+        <v>4447.11</v>
       </c>
       <c r="I13" s="33">
-        <v>4522.71</v>
+        <v>4518.27</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -2409,10 +2415,10 @@
         <v>548429.23</v>
       </c>
       <c r="H14" s="36">
-        <v>562837.52</v>
+        <v>562284.09</v>
       </c>
       <c r="I14" s="36">
-        <v>571842.92</v>
+        <v>571280.64</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2438,10 +2444,10 @@
         <v>4337.53</v>
       </c>
       <c r="H15" s="33">
-        <v>4451.49</v>
+        <v>4447.11</v>
       </c>
       <c r="I15" s="33">
-        <v>4522.71</v>
+        <v>4518.27</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -2467,10 +2473,10 @@
         <v>548429.23</v>
       </c>
       <c r="H16" s="36">
-        <v>562837.52</v>
+        <v>562284.09</v>
       </c>
       <c r="I16" s="36">
-        <v>571842.92</v>
+        <v>571280.64</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -2496,10 +2502,10 @@
         <v>4801.52</v>
       </c>
       <c r="H17" s="33">
-        <v>4923.5</v>
+        <v>4918.66</v>
       </c>
       <c r="I17" s="33">
-        <v>5002.28</v>
+        <v>4997.36</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -2525,10 +2531,10 @@
         <v>605050</v>
       </c>
       <c r="H18" s="36">
-        <v>620420.85</v>
+        <v>619810.8</v>
       </c>
       <c r="I18" s="36">
-        <v>630347.58</v>
+        <v>629727.77</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -2554,10 +2560,10 @@
         <v>4064.08</v>
       </c>
       <c r="H19" s="33">
-        <v>4174.62</v>
+        <v>4170.52</v>
       </c>
       <c r="I19" s="33">
-        <v>4241.42</v>
+        <v>4237.25</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -2583,10 +2589,10 @@
         <v>498582.06</v>
       </c>
       <c r="H20" s="36">
-        <v>512142.96</v>
+        <v>511639.37</v>
       </c>
       <c r="I20" s="36">
-        <v>520337.24</v>
+        <v>519825.6</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -2612,10 +2618,10 @@
         <v>4337.53</v>
       </c>
       <c r="H21" s="33">
-        <v>4451.49</v>
+        <v>4447.11</v>
       </c>
       <c r="I21" s="33">
-        <v>4522.71</v>
+        <v>4518.27</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2641,10 +2647,10 @@
         <v>548429.23</v>
       </c>
       <c r="H22" s="36">
-        <v>562837.52</v>
+        <v>562284.09</v>
       </c>
       <c r="I22" s="36">
-        <v>571842.92</v>
+        <v>571280.64</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
@@ -2976,7 +2982,7 @@
   <sheetPr>
     <tabColor rgb="FF37474F"/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
@@ -3016,15 +3022,15 @@
         <v>167</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" s="43" t="s">
         <v>168</v>
-      </c>
-      <c r="B7" s="43" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -3069,23 +3075,31 @@
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B13" s="43" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="B15" s="6"/>
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="B14" s="45" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1"/>
@@ -3097,6 +3111,7 @@
     <hyperlink ref="B11" r:id="rId7"/>
     <hyperlink ref="B12" r:id="rId8"/>
     <hyperlink ref="B13" r:id="rId9"/>
+    <hyperlink ref="B14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
ventas: las 5 calculadoras más usadas cierran la venta con su propio producto
- Planillas de Comercio, UOCRA y Casas Particulares: oferta dentro de la calculadora con la
  hoja armada con los números de la persona; la planilla comprada llega con esos datos
  cargados (viajan en la metadata del pago de MP, con consentimiento en el diálogo).
- Producto nuevo: Planilla de alquileres 2026 ($9.900) para dueños: contratos, IPC oficial
  embebido, cronograma de ajustes, recibo y aviso de aumento.
- Producto nuevo: Informe de cuota alimentaria ($4.900), documento A4 imprimible para la
  mediación, con la canasta de crianza del INDEC.
- Landings rediseñadas, privacidad actualizada, cupo y validación en las rutas de entrega,
  fórmulas de Comercio y UOCRA sin el «=» que hacía que Excel ofreciera reparar el archivo,
  citas del CCyC corregidas (659/666), sin anuncios en las páginas que venden.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-casas-particulares-2026.xlsx
+++ b/private/planilla-casas-particulares-2026.xlsx
@@ -97,244 +97,244 @@
     <t>Mes a liquidar</t>
   </si>
   <si>
+    <t>octubre de 2026</t>
+  </si>
+  <si>
+    <t>Categoría</t>
+  </si>
+  <si>
+    <t>Personal para tareas generales</t>
+  </si>
+  <si>
+    <t>Modalidad</t>
+  </si>
+  <si>
+    <t>Con retiro</t>
+  </si>
+  <si>
+    <t>Horas que trabaja por semana (en tu casa)</t>
+  </si>
+  <si>
+    <t>¿Zona desfavorable (Patagonia)?</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Horas extras del mes en días comunes</t>
+  </si>
+  <si>
+    <t>Horas extras sábado desde las 13, domingo o feriado</t>
+  </si>
+  <si>
+    <t>Condición de la trabajadora (para ARCA)</t>
+  </si>
+  <si>
+    <t>Mayor de 18 años</t>
+  </si>
+  <si>
+    <t>Chequeo</t>
+  </si>
+  <si>
+    <t>SUELDO DEL MES</t>
+  </si>
+  <si>
+    <t>Valor de la hora</t>
+  </si>
+  <si>
+    <t>Mínimo mensual (jornada completa de 48 h)</t>
+  </si>
+  <si>
+    <t>Horas trabajadas en el mes</t>
+  </si>
+  <si>
+    <t>Sueldo por las horas trabajadas</t>
+  </si>
+  <si>
+    <t>Básico del mes</t>
+  </si>
+  <si>
+    <t>Horas extras comunes (+50%)</t>
+  </si>
+  <si>
+    <t>Horas extras fin de semana y feriados (+100%)</t>
+  </si>
+  <si>
+    <t>TOTAL A PAGARLE ESTE MES</t>
+  </si>
+  <si>
+    <t>Aguinaldo que va generando (50%)</t>
+  </si>
+  <si>
+    <t>LO QUE LE PAGÁS A ARCA (aportes, contribuciones y ART)</t>
+  </si>
+  <si>
+    <t>Rango de horas para ARCA</t>
+  </si>
+  <si>
+    <t>Pago mensual a ARCA por esta trabajadora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  · de eso, cuota de la ART</t>
+  </si>
+  <si>
+    <t>Falta para que tenga obra social</t>
+  </si>
+  <si>
+    <t>Falta para que le compute la jubilación</t>
+  </si>
+  <si>
+    <t>COSTO TOTAL DEL MES (sueldo + ARCA)</t>
+  </si>
+  <si>
+    <t>* Importes mínimos legales. Si pactaron un sueldo mayor, se paga el pactado.</t>
+  </si>
+  <si>
+    <t>* Los pagos de los aportes son siempre a mes vencido: cada mes se paga por lo trabajado en el mes anterior. La excepción es la ART, que se paga a mes en curso.</t>
+  </si>
+  <si>
+    <t>* «Falta para…» aparece con menos de 16 horas semanales: pagás en regla, pero sin completar esa diferencia la trabajadora no accede a la obra social y ese mes no le computa para jubilarse. La diferencia la puede pagar ella o la pueden acordar.</t>
+  </si>
+  <si>
+    <t>Pagos del año 2026 — aguinaldo y vacaciones</t>
+  </si>
+  <si>
+    <t>Mes</t>
+  </si>
+  <si>
+    <t>Sueldo pagado</t>
+  </si>
+  <si>
+    <t>Pagado a ARCA</t>
+  </si>
+  <si>
+    <t>Notas</t>
+  </si>
+  <si>
+    <t>Enero 2026</t>
+  </si>
+  <si>
+    <t>Febrero 2026</t>
+  </si>
+  <si>
+    <t>Marzo 2026</t>
+  </si>
+  <si>
+    <t>Abril 2026</t>
+  </si>
+  <si>
+    <t>Mayo 2026</t>
+  </si>
+  <si>
+    <t>Junio 2026</t>
+  </si>
+  <si>
+    <t>Julio 2026</t>
+  </si>
+  <si>
+    <t>Agosto 2026</t>
+  </si>
+  <si>
+    <t>Septiembre 2026</t>
+  </si>
+  <si>
+    <t>Octubre 2026</t>
+  </si>
+  <si>
+    <t>Noviembre 2026</t>
+  </si>
+  <si>
+    <t>Diciembre 2026</t>
+  </si>
+  <si>
+    <t>AGUINALDO (Ley 26.844, art. 26)</t>
+  </si>
+  <si>
+    <t>Aguinaldo de junio (1er semestre)</t>
+  </si>
+  <si>
+    <t>Aguinaldo de diciembre (2do semestre)</t>
+  </si>
+  <si>
+    <t>Total pagado en sueldos en el año</t>
+  </si>
+  <si>
+    <t>Total pagado a ARCA en el año</t>
+  </si>
+  <si>
+    <t>VACACIONES (Ley 26.844, art. 29)</t>
+  </si>
+  <si>
+    <t>Antigüedad al 31 de diciembre (años)</t>
+  </si>
+  <si>
+    <t>Días de vacaciones que le corresponden</t>
+  </si>
+  <si>
+    <t>* El aguinaldo es el 50% del MEJOR sueldo del semestre, no el promedio. Si trabajó solo una parte del semestre, corresponde en proporción al tiempo trabajado: para ese caso usá calcular.ar/aguinaldo.</t>
+  </si>
+  <si>
+    <t>* Con menos de 6 meses de antigüedad no hay licencia completa: corresponde un día de descanso cada 20 días trabajados (Ley 26.844, art. 30).</t>
+  </si>
+  <si>
+    <t>Recibo de sueldo — Personal de Casas Particulares</t>
+  </si>
+  <si>
+    <t>Modelo para imprimir por duplicado: una copia firmada queda para cada parte. Las celdas amarillas se completan una sola vez.</t>
+  </si>
+  <si>
+    <t>Empleador/a (nombre y apellido)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>CUIL/CUIT del empleador/a</t>
+  </si>
+  <si>
+    <t>Trabajador/a (nombre y apellido)</t>
+  </si>
+  <si>
+    <t>CUIL del trabajador/a</t>
+  </si>
+  <si>
+    <t>Período</t>
+  </si>
+  <si>
+    <t>Horas semanales</t>
+  </si>
+  <si>
+    <t>Básico</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Fecha de pago</t>
+  </si>
+  <si>
+    <t>Recibí conforme el importe total indicado.</t>
+  </si>
+  <si>
+    <t>Firma del trabajador/a</t>
+  </si>
+  <si>
+    <t>Firma del empleador/a</t>
+  </si>
+  <si>
+    <t>Escala oficial — Personal de Casas Particulares 2026 (Resolución CNTCP 6/2026)</t>
+  </si>
+  <si>
+    <t>Clave</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>agosto de 2026</t>
+  </si>
+  <si>
     <t>septiembre de 2026</t>
-  </si>
-  <si>
-    <t>Categoría</t>
-  </si>
-  <si>
-    <t>Personal para tareas generales</t>
-  </si>
-  <si>
-    <t>Modalidad</t>
-  </si>
-  <si>
-    <t>Con retiro</t>
-  </si>
-  <si>
-    <t>Horas que trabaja por semana (en tu casa)</t>
-  </si>
-  <si>
-    <t>¿Zona desfavorable (Patagonia)?</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Horas extras del mes en días comunes</t>
-  </si>
-  <si>
-    <t>Horas extras sábado desde las 13, domingo o feriado</t>
-  </si>
-  <si>
-    <t>Condición de la trabajadora (para ARCA)</t>
-  </si>
-  <si>
-    <t>Mayor de 18 años</t>
-  </si>
-  <si>
-    <t>Chequeo</t>
-  </si>
-  <si>
-    <t>SUELDO DEL MES</t>
-  </si>
-  <si>
-    <t>Valor de la hora</t>
-  </si>
-  <si>
-    <t>Mínimo mensual (jornada completa de 48 h)</t>
-  </si>
-  <si>
-    <t>Horas trabajadas en el mes</t>
-  </si>
-  <si>
-    <t>Sueldo por las horas trabajadas</t>
-  </si>
-  <si>
-    <t>Básico del mes</t>
-  </si>
-  <si>
-    <t>Horas extras comunes (+50%)</t>
-  </si>
-  <si>
-    <t>Horas extras fin de semana y feriados (+100%)</t>
-  </si>
-  <si>
-    <t>TOTAL A PAGARLE ESTE MES</t>
-  </si>
-  <si>
-    <t>Aguinaldo que va generando (50%)</t>
-  </si>
-  <si>
-    <t>LO QUE LE PAGÁS A ARCA (aportes, contribuciones y ART)</t>
-  </si>
-  <si>
-    <t>Rango de horas para ARCA</t>
-  </si>
-  <si>
-    <t>Pago mensual a ARCA por esta trabajadora</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · de eso, cuota de la ART</t>
-  </si>
-  <si>
-    <t>Falta para que tenga obra social</t>
-  </si>
-  <si>
-    <t>Falta para que le compute la jubilación</t>
-  </si>
-  <si>
-    <t>COSTO TOTAL DEL MES (sueldo + ARCA)</t>
-  </si>
-  <si>
-    <t>* Importes mínimos legales. Si pactaron un sueldo mayor, se paga el pactado.</t>
-  </si>
-  <si>
-    <t>* Los pagos de los aportes son siempre a mes vencido: cada mes se paga por lo trabajado en el mes anterior. La excepción es la ART, que se paga a mes en curso.</t>
-  </si>
-  <si>
-    <t>* «Falta para…» aparece con menos de 16 horas semanales: pagás en regla, pero sin completar esa diferencia la trabajadora no accede a la obra social y ese mes no le computa para jubilarse. La diferencia la puede pagar ella o la pueden acordar.</t>
-  </si>
-  <si>
-    <t>Pagos del año 2026 — aguinaldo y vacaciones</t>
-  </si>
-  <si>
-    <t>Mes</t>
-  </si>
-  <si>
-    <t>Sueldo pagado</t>
-  </si>
-  <si>
-    <t>Pagado a ARCA</t>
-  </si>
-  <si>
-    <t>Notas</t>
-  </si>
-  <si>
-    <t>Enero 2026</t>
-  </si>
-  <si>
-    <t>Febrero 2026</t>
-  </si>
-  <si>
-    <t>Marzo 2026</t>
-  </si>
-  <si>
-    <t>Abril 2026</t>
-  </si>
-  <si>
-    <t>Mayo 2026</t>
-  </si>
-  <si>
-    <t>Junio 2026</t>
-  </si>
-  <si>
-    <t>Julio 2026</t>
-  </si>
-  <si>
-    <t>Agosto 2026</t>
-  </si>
-  <si>
-    <t>Septiembre 2026</t>
-  </si>
-  <si>
-    <t>Octubre 2026</t>
-  </si>
-  <si>
-    <t>Noviembre 2026</t>
-  </si>
-  <si>
-    <t>Diciembre 2026</t>
-  </si>
-  <si>
-    <t>AGUINALDO (Ley 26.844, art. 26)</t>
-  </si>
-  <si>
-    <t>Aguinaldo de junio (1er semestre)</t>
-  </si>
-  <si>
-    <t>Aguinaldo de diciembre (2do semestre)</t>
-  </si>
-  <si>
-    <t>Total pagado en sueldos en el año</t>
-  </si>
-  <si>
-    <t>Total pagado a ARCA en el año</t>
-  </si>
-  <si>
-    <t>VACACIONES (Ley 26.844, art. 29)</t>
-  </si>
-  <si>
-    <t>Antigüedad al 31 de diciembre (años)</t>
-  </si>
-  <si>
-    <t>Días de vacaciones que le corresponden</t>
-  </si>
-  <si>
-    <t>* El aguinaldo es el 50% del MEJOR sueldo del semestre, no el promedio. Si trabajó solo una parte del semestre, corresponde en proporción al tiempo trabajado: para ese caso usá calcular.ar/aguinaldo.</t>
-  </si>
-  <si>
-    <t>* Con menos de 6 meses de antigüedad no hay licencia completa: corresponde un día de descanso cada 20 días trabajados (Ley 26.844, art. 30).</t>
-  </si>
-  <si>
-    <t>Recibo de sueldo — Personal de Casas Particulares</t>
-  </si>
-  <si>
-    <t>Modelo para imprimir por duplicado: una copia firmada queda para cada parte. Las celdas amarillas se completan una sola vez.</t>
-  </si>
-  <si>
-    <t>Empleador/a (nombre y apellido)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>CUIL/CUIT del empleador/a</t>
-  </si>
-  <si>
-    <t>Trabajador/a (nombre y apellido)</t>
-  </si>
-  <si>
-    <t>CUIL del trabajador/a</t>
-  </si>
-  <si>
-    <t>Período</t>
-  </si>
-  <si>
-    <t>Horas semanales</t>
-  </si>
-  <si>
-    <t>Básico</t>
-  </si>
-  <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>Fecha de pago</t>
-  </si>
-  <si>
-    <t>Recibí conforme el importe total indicado.</t>
-  </si>
-  <si>
-    <t>Firma del trabajador/a</t>
-  </si>
-  <si>
-    <t>Firma del empleador/a</t>
-  </si>
-  <si>
-    <t>Escala oficial — Personal de Casas Particulares 2026 (Resolución CNTCP 6/2026)</t>
-  </si>
-  <si>
-    <t>Clave</t>
-  </si>
-  <si>
-    <t>Valor</t>
-  </si>
-  <si>
-    <t>agosto de 2026</t>
-  </si>
-  <si>
-    <t>octubre de 2026</t>
   </si>
   <si>
     <t>noviembre de 2026</t>
@@ -2081,10 +2081,10 @@
         <v>104</v>
       </c>
       <c r="F2" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="G2" s="30" t="s">
         <v>26</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>105</v>
       </c>
       <c r="H2" s="30" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
casas particulares: adicional por antigüedad del 1% por año (Res. CNTCP 2/2021, art. 3)
Calculadora, planilla .xlsx (fila nueva en el Liquidador y en el recibo), vista
previa y prefill. Los años se cuentan desde el 1/9/2020 sin efecto retroactivo:
tope de 6 años desde septiembre de 2026. check_planilla_casas compara 105 casos
de antigüedad contra el motor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-casas-particulares-2026.xlsx
+++ b/private/planilla-casas-particulares-2026.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="189">
   <si>
     <t>Cómo usar esta planilla</t>
   </si>
@@ -25,7 +25,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>Andá a la hoja «Liquidador». Completá solo las celdas amarillas: mes, categoría, modalidad, horas por semana, zona, horas extras y la condición de la persona que trabaja en tu casa.</t>
+    <t>Andá a la hoja «Liquidador». Completá solo las celdas amarillas: mes, categoría, modalidad, horas por semana, zona, años de antigüedad, horas extras y la condición de la persona que trabaja en tu casa.</t>
   </si>
   <si>
     <t>2</t>
@@ -64,6 +64,9 @@
     <t>•  Zona desfavorable: 31% sobre el mínimo de cada categoría desde el 1 de abril de 2026, en La Pampa, Río Negro, Chubut, Neuquén, Santa Cruz, Tierra del Fuego, Antártida e Islas del Atlántico Sur y el partido de Patagones.</t>
   </si>
   <si>
+    <t>•  Antigüedad: 1% del básico por cada año (art. 3 de la Resolución CNTCP 2/2021). Los años se cuentan desde el 1 de septiembre de 2020, sin efecto retroactivo: aunque haya entrado antes, en octubre de 2026 suma como máximo 6 años. La planilla aplica ese tope sola.</t>
+  </si>
+  <si>
     <t>•  Aguinaldo: 50% de la mayor remuneración mensual del semestre (Ley 26.844, art. 26). Se paga en junio y en diciembre.</t>
   </si>
   <si>
@@ -121,6 +124,9 @@
     <t>No</t>
   </si>
   <si>
+    <t>Años completos de antigüedad</t>
+  </si>
+  <si>
     <t>Horas extras del mes en días comunes</t>
   </si>
   <si>
@@ -154,6 +160,9 @@
     <t>Básico del mes</t>
   </si>
   <si>
+    <t>Adicional por antigüedad (1% por año)</t>
+  </si>
+  <si>
     <t>Horas extras comunes (+50%)</t>
   </si>
   <si>
@@ -196,6 +205,9 @@
     <t>* «Falta para…» aparece con menos de 16 horas semanales: pagás en regla, pero sin completar esa diferencia la trabajadora no accede a la obra social y ese mes no le computa para jubilarse. La diferencia la puede pagar ella o la pueden acordar.</t>
   </si>
   <si>
+    <t>* Antigüedad (art. 3 de la Resolución CNTCP 2/2021): 1% del básico por año completo, contado desde el 1 de septiembre de 2020 sin efecto retroactivo. Si cargás más años de los que se pueden contar en el mes elegido, la planilla toma el máximo. Para vacaciones e indemnización vale la antigüedad completa.</t>
+  </si>
+  <si>
     <t>Pagos del año 2026 — aguinaldo y vacaciones</t>
   </si>
   <si>
@@ -533,6 +545,12 @@
   </si>
   <si>
     <t>https://www.argentina.gob.ar/normativa/426540_res4-4_pdf/archivo</t>
+  </si>
+  <si>
+    <t>Resolución CNTCP 2/2021: crea el adicional por antigüedad</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/246035/20210625</t>
   </si>
   <si>
     <t>Ley 26.844: Régimen Especial para el Personal de Casas Particulares</t>
@@ -1211,7 +1229,7 @@
   <sheetPr>
     <tabColor rgb="FFF57C00"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1315,17 +1333,22 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" ht="44" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    <row r="19" ht="36" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="6"/>
+    </row>
+    <row r="21" ht="44" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1337,7 +1360,7 @@
   <sheetPr>
     <tabColor rgb="FF1B5E20"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -1348,28 +1371,28 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5">
         <f>MATCH(B5,'Escala 2026'!$E$2:$I$2,0)</f>
@@ -1377,10 +1400,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6">
         <f>CONCATENATE("H|",B6,"|",B7)</f>
@@ -1388,10 +1411,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7">
         <f>IFERROR(INDEX('Escala 2026'!$E$3:$I$22,MATCH(D6,'Escala 2026'!$A$3:$A$22,0),D5),0)</f>
@@ -1399,7 +1422,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" s="11">
         <v>20</v>
@@ -1410,10 +1433,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9">
         <f>IFERROR(INDEX('Escala 2026'!$E$3:$I$22,MATCH(D8,'Escala 2026'!$A$3:$A$22,0),D5),0)</f>
@@ -1421,7 +1444,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="11">
         <v>0</v>
@@ -1432,7 +1455,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="11">
         <v>0</v>
@@ -1443,10 +1466,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="10" t="s">
         <v>37</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0</v>
       </c>
       <c r="D12">
         <f>IF(MAX(B8,0)&gt;=16,"16 horas semanales o más",IF(MAX(B8,0)&gt;=12,"Desde 12 a menos de 16 horas semanales","Menos de 12 horas semanales"))</f>
@@ -1456,184 +1479,217 @@
       <c r="A13" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13">
+        <f>CONCATENATE(B13,"|",D12)</f>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="12">
         <f>IF(D7=0,"Esa combinación no existe en la escala oficial: los caseros son siempre sin retiro.","OK")</f>
       </c>
-      <c r="D13">
-        <f>CONCATENATE(B12,"|",D12)</f>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="4"/>
       <c r="D14">
-        <f>CONCATENATE(B12,"|","16 horas semanales o más")</f>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="14">
+        <f>CONCATENATE(B13,"|","16 horas semanales o más")</f>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="D15">
+        <f>IFERROR(CHOOSE(D5,5,6,6,6,6),0)</f>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="14">
         <f>IF(D7=0,0,ROUND(D7*D10,2))</f>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="14">
-        <f>ROUND(D9*D10,2)</f>
+      <c r="D16">
+        <f>MIN(MAX(INT(B10),0),D15)</f>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="15">
-        <f>ROUND(D11*52/12,2)</f>
+        <v>43</v>
+      </c>
+      <c r="B17" s="14">
+        <f>ROUND(D9*D10,2)</f>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="14">
-        <f>ROUND(B15*B17,2)</f>
+        <v>44</v>
+      </c>
+      <c r="B18" s="15">
+        <f>ROUND(D11*52/12,2)</f>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" s="14">
-        <f>IF(D11&gt;=48,MAX(B18,B16),B18)</f>
+        <f>ROUND(B16*B18,2)</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="14">
-        <f>ROUND(MAX(B10,0)*B15*1.5,2)</f>
+        <f>IF(D11&gt;=48,MAX(B19,B17),B19)</f>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="14">
-        <f>ROUND(MAX(B11,0)*B15*2,2)</f>
+        <f>ROUND(B20*D16*1/100,2)</f>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="17">
-        <f>ROUND(B19+B20+B21,2)</f>
+      <c r="A22" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="14">
+        <f>ROUND(MAX(B11,0)*B16*1.5,2)</f>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" s="14">
-        <f>ROUND(B22/2,2)</f>
-      </c>
-    </row>
-    <row r="24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+        <f>ROUND(MAX(B12,0)*B16*2,2)</f>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="17">
+        <f>ROUND(B20+B21+B22+B23,2)</f>
+      </c>
+    </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" s="18">
-        <f>D12</f>
-      </c>
-    </row>
+      <c r="A25" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="14">
+        <f>ROUND(B24/2,2)</f>
+      </c>
+    </row>
+    <row r="26" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="14">
-        <f>IFERROR(INDEX('Aportes ARCA'!$D$3:$D$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
-      </c>
+      <c r="A27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="14">
-        <f>IFERROR(INDEX('Aportes ARCA'!$G$3:$G$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
+        <v>53</v>
+      </c>
+      <c r="B28" s="18">
+        <f>D12</f>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B29" s="14">
-        <f>MAX(0,ROUND(IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D14,'Aportes ARCA'!$A$3:$A$11,0)),0)-IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0),2))</f>
+        <f>IFERROR(INDEX('Aportes ARCA'!$D$3:$D$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="14">
+        <f>IFERROR(INDEX('Aportes ARCA'!$G$3:$G$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="14">
+        <f>MAX(0,ROUND(IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D14,'Aportes ARCA'!$A$3:$A$11,0)),0)-IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0),2))</f>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="14">
         <f>MAX(0,ROUND(IFERROR(INDEX('Aportes ARCA'!$F$3:$F$11,MATCH(D14,'Aportes ARCA'!$A$3:$A$11,0)),0)-IFERROR(INDEX('Aportes ARCA'!$F$3:$F$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0),2))</f>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B31" s="17">
-        <f>ROUND(B22+B27,2)</f>
-      </c>
-    </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B33" s="6"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="6"/>
-    </row>
-    <row r="35" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="17">
+        <f>ROUND(B24+B29,2)</f>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B35" s="6"/>
     </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="6"/>
+    </row>
+    <row r="37" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="6"/>
+    </row>
+    <row r="38" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
   </mergeCells>
-  <dataValidations count="7">
-    <dataValidation type="decimal" showErrorMessage="1" error="Entre 0 y 200 horas." sqref="B10:B11">
+  <dataValidations count="8">
+    <dataValidation type="whole" showErrorMessage="1" error="Ingresá los años completos que lleva trabajando en tu casa (entre 0 y 60)." sqref="B10">
+      <formula1>0</formula1>
+      <formula2>60</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" showErrorMessage="1" error="Entre 0 y 200 horas." sqref="B11:B12">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" error="Elegí una condición de la lista." sqref="B12">
+    <dataValidation type="list" showErrorMessage="1" error="Elegí una condición de la lista." sqref="B13">
       <formula1>"Mayor de 18 años,De 16 o 17 años,Jubilado/a"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B5">
@@ -1673,7 +1729,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1681,21 +1737,21 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B4" s="21"/>
       <c r="C4" s="21"/>
@@ -1703,7 +1759,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -1711,7 +1767,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -1719,7 +1775,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" s="21"/>
       <c r="C7" s="21"/>
@@ -1727,7 +1783,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -1735,7 +1791,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -1743,7 +1799,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
@@ -1751,7 +1807,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
@@ -1759,7 +1815,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="21"/>
@@ -1767,7 +1823,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="21"/>
@@ -1775,7 +1831,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
@@ -1783,7 +1839,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="21"/>
@@ -1791,13 +1847,13 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B16" s="4"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B17" s="14">
         <f>ROUND(MAX(B4:B9)/2,2)</f>
@@ -1805,7 +1861,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B18" s="14">
         <f>ROUND(MAX(B10:B15)/2,2)</f>
@@ -1813,7 +1869,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B19" s="14">
         <f>SUM(B4:B15)</f>
@@ -1821,7 +1877,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B20" s="14">
         <f>SUM(C4:C15)</f>
@@ -1829,13 +1885,13 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B22" s="4"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B23" s="23">
         <v>1</v>
@@ -1843,7 +1899,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B24" s="24">
         <f>IF(B23&lt;=5,14,IF(B23&lt;=10,21,IF(B23&lt;=20,28,35)))</f>
@@ -1851,7 +1907,7 @@
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1859,7 +1915,7 @@
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1890,7 +1946,7 @@
     <tabColor rgb="FF455A64"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1899,51 +1955,51 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B1" s="25"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B2" s="6"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B8" s="13">
         <f>'Liquidador'!B5</f>
@@ -1951,7 +2007,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="13">
         <f>'Liquidador'!B6</f>
@@ -1959,7 +2015,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="13">
         <f>'Liquidador'!B7</f>
@@ -1967,7 +2023,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B11" s="26">
         <f>'Liquidador'!B8</f>
@@ -1975,55 +2031,63 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B12" s="14">
-        <f>'Liquidador'!B19</f>
+        <f>'Liquidador'!B20</f>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B13" s="14">
-        <f>'Liquidador'!B20</f>
+        <f>'Liquidador'!B21</f>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B14" s="14">
-        <f>'Liquidador'!B21</f>
+        <f>'Liquidador'!B22</f>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" s="17">
-        <f>'Liquidador'!B22</f>
+        <v>49</v>
+      </c>
+      <c r="B15" s="14">
+        <f>'Liquidador'!B23</f>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="B22" s="28" t="s">
         <v>100</v>
+      </c>
+      <c r="B16" s="17">
+        <f>'Liquidador'!B24</f>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2053,7 +2117,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -2066,45 +2130,45 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="G2" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>26</v>
-      </c>
       <c r="H2" s="30" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I2" s="30" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E3" s="33">
         <v>4523.11</v>
@@ -2124,16 +2188,16 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E4" s="36">
         <v>564246.7</v>
@@ -2153,16 +2217,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="32" t="s">
-        <v>109</v>
-      </c>
       <c r="C5" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D5" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E5" s="33">
         <v>4920.89</v>
@@ -2182,16 +2246,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D6" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E6" s="36">
         <v>624313.9</v>
@@ -2211,16 +2275,16 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E7" s="33">
         <v>4303.5</v>
@@ -2240,16 +2304,16 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E8" s="36">
         <v>526829.56</v>
@@ -2269,16 +2333,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C9" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D9" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E9" s="33">
         <v>4684.53</v>
@@ -2298,16 +2362,16 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E10" s="36">
         <v>582283.26</v>
@@ -2327,16 +2391,16 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E11" s="33"/>
       <c r="F11" s="33"/>
@@ -2346,16 +2410,16 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E12" s="36"/>
       <c r="F12" s="36"/>
@@ -2365,16 +2429,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C13" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D13" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E13" s="33">
         <v>4072.38</v>
@@ -2394,16 +2458,16 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E14" s="36">
         <v>514903.51</v>
@@ -2423,16 +2487,16 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E15" s="33">
         <v>4072.38</v>
@@ -2452,16 +2516,16 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E16" s="36">
         <v>514903.51</v>
@@ -2481,16 +2545,16 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B17" s="32" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C17" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D17" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E17" s="33">
         <v>4520.15</v>
@@ -2510,16 +2574,16 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="34" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E18" s="36">
         <v>569593.41</v>
@@ -2539,16 +2603,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E19" s="33">
         <v>3804.66</v>
@@ -2568,16 +2632,16 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="34" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C20" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E20" s="36">
         <v>466756.24</v>
@@ -2597,16 +2661,16 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C21" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D21" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E21" s="33">
         <v>4072.38</v>
@@ -2626,16 +2690,16 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="34" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D22" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E22" s="36">
         <v>514903.51</v>
@@ -2655,7 +2719,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -2668,7 +2732,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -2705,7 +2769,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -2716,36 +2780,36 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="38" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D2" s="38" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E2" s="38" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F2" s="38" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G2" s="38" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D3" s="33">
         <v>10569.57</v>
@@ -2762,13 +2826,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D4" s="36">
         <v>16627.46</v>
@@ -2785,13 +2849,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="32" t="s">
-        <v>144</v>
-      </c>
       <c r="C5" s="32" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D5" s="33">
         <v>44270.19</v>
@@ -2808,13 +2872,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D6" s="36">
         <v>9839.67</v>
@@ -2829,13 +2893,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B7" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C7" s="32" t="s">
         <v>151</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>147</v>
       </c>
       <c r="D7" s="33">
         <v>15167.98</v>
@@ -2850,13 +2914,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="35" t="s">
         <v>153</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>149</v>
       </c>
       <c r="D8" s="36">
         <v>42141.4</v>
@@ -2871,13 +2935,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D9" s="33">
         <v>8484.72</v>
@@ -2892,13 +2956,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D10" s="36">
         <v>12764.16</v>
@@ -2913,13 +2977,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D11" s="33">
         <v>18575.64</v>
@@ -2934,7 +2998,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -2945,7 +3009,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2956,7 +3020,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -2982,7 +3046,7 @@
   <sheetPr>
     <tabColor rgb="FF37474F"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
@@ -2991,115 +3055,123 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B1" s="39"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B2" s="40"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="42" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="44" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B9" s="43" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="44" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="42" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B11" s="43" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="44" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B12" s="45" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B13" s="43" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="44" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B14" s="45" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B16" s="6"/>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="42" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="43" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1"/>
@@ -3112,6 +3184,7 @@
     <hyperlink ref="B12" r:id="rId8"/>
     <hyperlink ref="B13" r:id="rId9"/>
     <hyperlink ref="B14" r:id="rId10"/>
+    <hyperlink ref="B15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Pendientes de calcular: SMVM en horas, fechas de pago, BE/NL, hreflang y antigüedad de casas particulares (#92)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/private/planilla-casas-particulares-2026.xlsx
+++ b/private/planilla-casas-particulares-2026.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="189">
   <si>
     <t>Cómo usar esta planilla</t>
   </si>
@@ -25,7 +25,7 @@
     <t>1</t>
   </si>
   <si>
-    <t>Andá a la hoja «Liquidador». Completá solo las celdas amarillas: mes, categoría, modalidad, horas por semana, zona, horas extras y la condición de la persona que trabaja en tu casa.</t>
+    <t>Andá a la hoja «Liquidador». Completá solo las celdas amarillas: mes, categoría, modalidad, horas por semana, zona, años de antigüedad, horas extras y la condición de la persona que trabaja en tu casa.</t>
   </si>
   <si>
     <t>2</t>
@@ -64,6 +64,9 @@
     <t>•  Zona desfavorable: 31% sobre el mínimo de cada categoría desde el 1 de abril de 2026, en La Pampa, Río Negro, Chubut, Neuquén, Santa Cruz, Tierra del Fuego, Antártida e Islas del Atlántico Sur y el partido de Patagones.</t>
   </si>
   <si>
+    <t>•  Antigüedad: 1% del básico por cada año (art. 3 de la Resolución CNTCP 2/2021). Los años se cuentan desde el 1 de septiembre de 2020, sin efecto retroactivo: aunque haya entrado antes, en octubre de 2026 suma como máximo 6 años. La planilla aplica ese tope sola.</t>
+  </si>
+  <si>
     <t>•  Aguinaldo: 50% de la mayor remuneración mensual del semestre (Ley 26.844, art. 26). Se paga en junio y en diciembre.</t>
   </si>
   <si>
@@ -121,6 +124,9 @@
     <t>No</t>
   </si>
   <si>
+    <t>Años completos de antigüedad</t>
+  </si>
+  <si>
     <t>Horas extras del mes en días comunes</t>
   </si>
   <si>
@@ -154,6 +160,9 @@
     <t>Básico del mes</t>
   </si>
   <si>
+    <t>Adicional por antigüedad (1% por año)</t>
+  </si>
+  <si>
     <t>Horas extras comunes (+50%)</t>
   </si>
   <si>
@@ -196,6 +205,9 @@
     <t>* «Falta para…» aparece con menos de 16 horas semanales: pagás en regla, pero sin completar esa diferencia la trabajadora no accede a la obra social y ese mes no le computa para jubilarse. La diferencia la puede pagar ella o la pueden acordar.</t>
   </si>
   <si>
+    <t>* Antigüedad (art. 3 de la Resolución CNTCP 2/2021): 1% del básico por año completo, contado desde el 1 de septiembre de 2020 sin efecto retroactivo. Si cargás más años de los que se pueden contar en el mes elegido, la planilla toma el máximo. Para vacaciones e indemnización vale la antigüedad completa.</t>
+  </si>
+  <si>
     <t>Pagos del año 2026 — aguinaldo y vacaciones</t>
   </si>
   <si>
@@ -533,6 +545,12 @@
   </si>
   <si>
     <t>https://www.argentina.gob.ar/normativa/426540_res4-4_pdf/archivo</t>
+  </si>
+  <si>
+    <t>Resolución CNTCP 2/2021: crea el adicional por antigüedad</t>
+  </si>
+  <si>
+    <t>https://www.boletinoficial.gob.ar/detalleAviso/primera/246035/20210625</t>
   </si>
   <si>
     <t>Ley 26.844: Régimen Especial para el Personal de Casas Particulares</t>
@@ -1211,7 +1229,7 @@
   <sheetPr>
     <tabColor rgb="FFF57C00"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1315,17 +1333,22 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" ht="44" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    <row r="19" ht="36" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="6"/>
+    </row>
+    <row r="21" ht="44" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1337,7 +1360,7 @@
   <sheetPr>
     <tabColor rgb="FF1B5E20"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -1348,28 +1371,28 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5">
         <f>MATCH(B5,'Escala 2026'!$E$2:$I$2,0)</f>
@@ -1377,10 +1400,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6">
         <f>CONCATENATE("H|",B6,"|",B7)</f>
@@ -1388,10 +1411,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7">
         <f>IFERROR(INDEX('Escala 2026'!$E$3:$I$22,MATCH(D6,'Escala 2026'!$A$3:$A$22,0),D5),0)</f>
@@ -1399,7 +1422,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" s="11">
         <v>20</v>
@@ -1410,10 +1433,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9">
         <f>IFERROR(INDEX('Escala 2026'!$E$3:$I$22,MATCH(D8,'Escala 2026'!$A$3:$A$22,0),D5),0)</f>
@@ -1421,7 +1444,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="11">
         <v>0</v>
@@ -1432,7 +1455,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="11">
         <v>0</v>
@@ -1443,10 +1466,10 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="10" t="s">
         <v>37</v>
+      </c>
+      <c r="B12" s="11">
+        <v>0</v>
       </c>
       <c r="D12">
         <f>IF(MAX(B8,0)&gt;=16,"16 horas semanales o más",IF(MAX(B8,0)&gt;=12,"Desde 12 a menos de 16 horas semanales","Menos de 12 horas semanales"))</f>
@@ -1456,184 +1479,217 @@
       <c r="A13" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13">
+        <f>CONCATENATE(B13,"|",D12)</f>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="12">
         <f>IF(D7=0,"Esa combinación no existe en la escala oficial: los caseros son siempre sin retiro.","OK")</f>
       </c>
-      <c r="D13">
-        <f>CONCATENATE(B12,"|",D12)</f>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="4"/>
       <c r="D14">
-        <f>CONCATENATE(B12,"|","16 horas semanales o más")</f>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="14">
+        <f>CONCATENATE(B13,"|","16 horas semanales o más")</f>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="D15">
+        <f>IFERROR(CHOOSE(D5,5,6,6,6,6),0)</f>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="14">
         <f>IF(D7=0,0,ROUND(D7*D10,2))</f>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="14">
-        <f>ROUND(D9*D10,2)</f>
+      <c r="D16">
+        <f>MIN(MAX(INT(B10),0),D15)</f>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="15">
-        <f>ROUND(D11*52/12,2)</f>
+        <v>43</v>
+      </c>
+      <c r="B17" s="14">
+        <f>ROUND(D9*D10,2)</f>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="14">
-        <f>ROUND(B15*B17,2)</f>
+        <v>44</v>
+      </c>
+      <c r="B18" s="15">
+        <f>ROUND(D11*52/12,2)</f>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" s="14">
-        <f>IF(D11&gt;=48,MAX(B18,B16),B18)</f>
+        <f>ROUND(B16*B18,2)</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20" s="14">
-        <f>ROUND(MAX(B10,0)*B15*1.5,2)</f>
+        <f>IF(D11&gt;=48,MAX(B19,B17),B19)</f>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="14">
-        <f>ROUND(MAX(B11,0)*B15*2,2)</f>
+        <f>ROUND(B20*D16*1/100,2)</f>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="17">
-        <f>ROUND(B19+B20+B21,2)</f>
+      <c r="A22" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="14">
+        <f>ROUND(MAX(B11,0)*B16*1.5,2)</f>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23" s="14">
-        <f>ROUND(B22/2,2)</f>
-      </c>
-    </row>
-    <row r="24" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+        <f>ROUND(MAX(B12,0)*B16*2,2)</f>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="17">
+        <f>ROUND(B20+B21+B22+B23,2)</f>
+      </c>
+    </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" s="18">
-        <f>D12</f>
-      </c>
-    </row>
+      <c r="A25" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="14">
+        <f>ROUND(B24/2,2)</f>
+      </c>
+    </row>
+    <row r="26" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="14">
-        <f>IFERROR(INDEX('Aportes ARCA'!$D$3:$D$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
-      </c>
+      <c r="A27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="4"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="14">
-        <f>IFERROR(INDEX('Aportes ARCA'!$G$3:$G$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
+        <v>53</v>
+      </c>
+      <c r="B28" s="18">
+        <f>D12</f>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B29" s="14">
-        <f>MAX(0,ROUND(IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D14,'Aportes ARCA'!$A$3:$A$11,0)),0)-IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0),2))</f>
+        <f>IFERROR(INDEX('Aportes ARCA'!$D$3:$D$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="14">
+        <f>IFERROR(INDEX('Aportes ARCA'!$G$3:$G$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0)</f>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="14">
+        <f>MAX(0,ROUND(IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D14,'Aportes ARCA'!$A$3:$A$11,0)),0)-IFERROR(INDEX('Aportes ARCA'!$E$3:$E$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0),2))</f>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="14">
         <f>MAX(0,ROUND(IFERROR(INDEX('Aportes ARCA'!$F$3:$F$11,MATCH(D14,'Aportes ARCA'!$A$3:$A$11,0)),0)-IFERROR(INDEX('Aportes ARCA'!$F$3:$F$11,MATCH(D13,'Aportes ARCA'!$A$3:$A$11,0)),0),2))</f>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B31" s="17">
-        <f>ROUND(B22+B27,2)</f>
-      </c>
-    </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B33" s="6"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="6"/>
-    </row>
-    <row r="35" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="17">
+        <f>ROUND(B24+B29,2)</f>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B35" s="6"/>
     </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="6"/>
+    </row>
+    <row r="37" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="6"/>
+    </row>
+    <row r="38" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
   </mergeCells>
-  <dataValidations count="7">
-    <dataValidation type="decimal" showErrorMessage="1" error="Entre 0 y 200 horas." sqref="B10:B11">
+  <dataValidations count="8">
+    <dataValidation type="whole" showErrorMessage="1" error="Ingresá los años completos que lleva trabajando en tu casa (entre 0 y 60)." sqref="B10">
+      <formula1>0</formula1>
+      <formula2>60</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" showErrorMessage="1" error="Entre 0 y 200 horas." sqref="B11:B12">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" error="Elegí una condición de la lista." sqref="B12">
+    <dataValidation type="list" showErrorMessage="1" error="Elegí una condición de la lista." sqref="B13">
       <formula1>"Mayor de 18 años,De 16 o 17 años,Jubilado/a"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Elegí un mes de la lista." sqref="B5">
@@ -1673,7 +1729,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1681,21 +1737,21 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B4" s="21"/>
       <c r="C4" s="21"/>
@@ -1703,7 +1759,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B5" s="21"/>
       <c r="C5" s="21"/>
@@ -1711,7 +1767,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -1719,7 +1775,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B7" s="21"/>
       <c r="C7" s="21"/>
@@ -1727,7 +1783,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -1735,7 +1791,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -1743,7 +1799,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
@@ -1751,7 +1807,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
@@ -1759,7 +1815,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="21"/>
@@ -1767,7 +1823,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="21"/>
@@ -1775,7 +1831,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
@@ -1783,7 +1839,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B15" s="21"/>
       <c r="C15" s="21"/>
@@ -1791,13 +1847,13 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B16" s="4"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B17" s="14">
         <f>ROUND(MAX(B4:B9)/2,2)</f>
@@ -1805,7 +1861,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B18" s="14">
         <f>ROUND(MAX(B10:B15)/2,2)</f>
@@ -1813,7 +1869,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B19" s="14">
         <f>SUM(B4:B15)</f>
@@ -1821,7 +1877,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B20" s="14">
         <f>SUM(C4:C15)</f>
@@ -1829,13 +1885,13 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B22" s="4"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B23" s="23">
         <v>1</v>
@@ -1843,7 +1899,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B24" s="24">
         <f>IF(B23&lt;=5,14,IF(B23&lt;=10,21,IF(B23&lt;=20,28,35)))</f>
@@ -1851,7 +1907,7 @@
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1859,7 +1915,7 @@
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1890,7 +1946,7 @@
     <tabColor rgb="FF455A64"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1899,51 +1955,51 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B1" s="25"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B2" s="6"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B8" s="13">
         <f>'Liquidador'!B5</f>
@@ -1951,7 +2007,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="13">
         <f>'Liquidador'!B6</f>
@@ -1959,7 +2015,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="13">
         <f>'Liquidador'!B7</f>
@@ -1967,7 +2023,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B11" s="26">
         <f>'Liquidador'!B8</f>
@@ -1975,55 +2031,63 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B12" s="14">
-        <f>'Liquidador'!B19</f>
+        <f>'Liquidador'!B20</f>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B13" s="14">
-        <f>'Liquidador'!B20</f>
+        <f>'Liquidador'!B21</f>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B14" s="14">
-        <f>'Liquidador'!B21</f>
+        <f>'Liquidador'!B22</f>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" s="17">
-        <f>'Liquidador'!B22</f>
+        <v>49</v>
+      </c>
+      <c r="B15" s="14">
+        <f>'Liquidador'!B23</f>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="B22" s="28" t="s">
         <v>100</v>
+      </c>
+      <c r="B16" s="17">
+        <f>'Liquidador'!B24</f>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="27" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -2053,7 +2117,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -2066,45 +2130,45 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="30" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="G2" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="30" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>26</v>
-      </c>
       <c r="H2" s="30" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I2" s="30" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E3" s="33">
         <v>4523.11</v>
@@ -2124,16 +2188,16 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E4" s="36">
         <v>564246.7</v>
@@ -2153,16 +2217,16 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="32" t="s">
-        <v>109</v>
-      </c>
       <c r="C5" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D5" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E5" s="33">
         <v>4920.89</v>
@@ -2182,16 +2246,16 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D6" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E6" s="36">
         <v>624313.9</v>
@@ -2211,16 +2275,16 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B7" s="32" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E7" s="33">
         <v>4303.5</v>
@@ -2240,16 +2304,16 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E8" s="36">
         <v>526829.56</v>
@@ -2269,16 +2333,16 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C9" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D9" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E9" s="33">
         <v>4684.53</v>
@@ -2298,16 +2362,16 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E10" s="36">
         <v>582283.26</v>
@@ -2327,16 +2391,16 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E11" s="33"/>
       <c r="F11" s="33"/>
@@ -2346,16 +2410,16 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="34" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E12" s="36"/>
       <c r="F12" s="36"/>
@@ -2365,16 +2429,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B13" s="32" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C13" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D13" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E13" s="33">
         <v>4072.38</v>
@@ -2394,16 +2458,16 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="34" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C14" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E14" s="36">
         <v>514903.51</v>
@@ -2423,16 +2487,16 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B15" s="32" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D15" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E15" s="33">
         <v>4072.38</v>
@@ -2452,16 +2516,16 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="34" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E16" s="36">
         <v>514903.51</v>
@@ -2481,16 +2545,16 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B17" s="32" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C17" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D17" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E17" s="33">
         <v>4520.15</v>
@@ -2510,16 +2574,16 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="34" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E18" s="36">
         <v>569593.41</v>
@@ -2539,16 +2603,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B19" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E19" s="33">
         <v>3804.66</v>
@@ -2568,16 +2632,16 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="34" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C20" s="35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E20" s="36">
         <v>466756.24</v>
@@ -2597,16 +2661,16 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B21" s="32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C21" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" s="32" t="s">
         <v>114</v>
-      </c>
-      <c r="D21" s="32" t="s">
-        <v>110</v>
       </c>
       <c r="E21" s="33">
         <v>4072.38</v>
@@ -2626,16 +2690,16 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="34" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="35" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D22" s="35" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E22" s="36">
         <v>514903.51</v>
@@ -2655,7 +2719,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -2668,7 +2732,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -2705,7 +2769,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B1" s="37"/>
       <c r="C1" s="37"/>
@@ -2716,36 +2780,36 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="38" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="38" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D2" s="38" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E2" s="38" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F2" s="38" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G2" s="38" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="31" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D3" s="33">
         <v>10569.57</v>
@@ -2762,13 +2826,13 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="34" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D4" s="36">
         <v>16627.46</v>
@@ -2785,13 +2849,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" s="32" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="32" t="s">
-        <v>144</v>
-      </c>
       <c r="C5" s="32" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D5" s="33">
         <v>44270.19</v>
@@ -2808,13 +2872,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="34" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D6" s="36">
         <v>9839.67</v>
@@ -2829,13 +2893,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="31" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B7" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C7" s="32" t="s">
         <v>151</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>147</v>
       </c>
       <c r="D7" s="33">
         <v>15167.98</v>
@@ -2850,13 +2914,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="35" t="s">
         <v>153</v>
-      </c>
-      <c r="B8" s="35" t="s">
-        <v>151</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>149</v>
       </c>
       <c r="D8" s="36">
         <v>42141.4</v>
@@ -2871,13 +2935,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="31" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B9" s="32" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D9" s="33">
         <v>8484.72</v>
@@ -2892,13 +2956,13 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D10" s="36">
         <v>12764.16</v>
@@ -2913,13 +2977,13 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="31" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B11" s="32" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D11" s="33">
         <v>18575.64</v>
@@ -2934,7 +2998,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -2945,7 +3009,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -2956,7 +3020,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -2982,7 +3046,7 @@
   <sheetPr>
     <tabColor rgb="FF37474F"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="62" customWidth="1"/>
@@ -2991,115 +3055,123 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B1" s="39"/>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B2" s="40"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B4" s="41" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="42" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="44" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="44" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B9" s="43" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="44" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="42" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B11" s="43" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="44" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B12" s="45" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B13" s="43" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="44" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="B14" s="45" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B16" s="6"/>
+        <v>187</v>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="42" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="43" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="B17" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1"/>
@@ -3112,6 +3184,7 @@
     <hyperlink ref="B12" r:id="rId8"/>
     <hyperlink ref="B13" r:id="rId9"/>
     <hyperlink ref="B14" r:id="rId10"/>
+    <hyperlink ref="B15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>